<commit_message>
Added new RDF data schemes and visual schemes for economy-table80-84, and fixed XLSX spreadsheets for economy-table81-83
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table81.xlsx
+++ b/sources/table_normalization/xlsx/economy-table81.xlsx
@@ -196,7 +196,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="yyyy/m/d;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy/m/d;@"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -264,10 +264,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -285,13 +285,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -303,7 +303,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>